<commit_message>
Reduz o escopo, foca o plano em Salvador e redesenha a contagem direta
- Plano de negócios para Salvador; concorrentes das 14 metrópoles da REGIC
  com mais de 100 avaliações servem de referência.
- Bloco B passa a coletar todas as avaliações com texto até "um mês atrás".
- Bloco C (histórico dos avaliadores) e comparação de modelos de A&B saem do
  escopo; emenda 2 ao registro prévio retira H2 e H4 e redefine H1
  (atendimento e ambiente × comida e bebida), conforme edição do autor no
  cronograma.
- Contagem direta: 2 visitas sorteadas e 2 de retorno 15 dias depois, do lado
  de fora, sem duração fixa, com leitura do número da NFC-e; script e
  planilha de sorteio refeitos com a mesma semente.
- Cronograma: cap. 5 em etapas (secundários primeiro, 5.3 após o Bloco A,
  5.2 após o fim da análise do Bloco B); cotações em Salvador na semana 4.
- Instruções, projeto, introdução e quadro de itens alinhados.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/textos/quadro de itens.xlsx
+++ b/textos/quadro de itens.xlsx
@@ -700,17 +700,17 @@
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Modelo de alimentos e bebidas (cozinha própria, parceria ou só bar)</t>
+          <t>Itens do cardápio que precisam de preparo (sem contar itens prontos, como balas, refrigerantes e água)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Nominal</t>
+          <t>Discreto</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Site, Instagram e cardápio digital de cada estabelecimento</t>
+          <t>Cardápio digital, site e Instagram de cada estabelecimento</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Definir o modelo de alimentos e bebidas da luderia</t>
+          <t>Medir a complexidade da cozinha dos concorrentes</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Google Maps: as 30 a 50 avaliações mais recentes com texto de cada estabelecimento</t>
+          <t>Google Maps: todas as avaliações com texto publicadas até "um mês atrás", por estabelecimento</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Google Maps: as 30 a 50 avaliações mais recentes com texto de cada estabelecimento</t>
+          <t>Google Maps: todas as avaliações com texto publicadas até "um mês atrás", por estabelecimento</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Google Maps: as 30 a 50 avaliações mais recentes com texto de cada estabelecimento</t>
+          <t>Google Maps: todas as avaliações com texto publicadas até "um mês atrás", por estabelecimento</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -834,12 +834,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Google Maps: as 30 a 50 avaliações mais recentes com texto de cada estabelecimento</t>
+          <t>Google Maps: todas as avaliações com texto publicadas até "um mês atrás", por estabelecimento</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Cálculo: avaliações do recorte ÷ intervalo entre a mais antiga e a mais recente</t>
+          <t>Cálculo: avaliações com texto do recorte ÷ duração da janela, a partir da data da coleta</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -854,27 +854,27 @@
       <c r="A13" s="5" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Nota centrada no avaliador</t>
+          <t>Entradas e saídas dos grupos</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Contínuo</t>
+          <t>Discreto</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Perfil público do avaliador no Google Maps, com o nome trocado por código</t>
+          <t>São Jogue, as duas unidades em Salvador</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Cópia do histórico de avaliações</t>
+          <t>Formulário de observação, do lado de fora: 2 visitas sorteadas e 2 de retorno 15 dias depois, com registro contínuo na porta</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Controlar o grau de exigência de cada avaliador</t>
+          <t>Medir o fluxo de pessoas por hora</t>
         </is>
       </c>
       <c r="G13" s="2" t="n"/>
@@ -884,27 +884,27 @@
       <c r="A14" s="5" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Categorias de lugares no histórico do avaliador</t>
+          <t>Número da nota fiscal (NFC-e) no início e no fim de cada visita</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Nominal</t>
+          <t>Discreto</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Perfil público do avaliador no Google Maps, com o nome trocado por código</t>
+          <t>São Jogue, as duas unidades em Salvador</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Cópia do histórico de avaliações</t>
+          <t>Registro da nota emitida em compra própria</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Traçar o perfil de consumo do público e indicar parcerias e localização</t>
+          <t>Medir as vendas entre a visita sorteada e a de retorno e as pessoas por nota</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -929,7 +929,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Formulário de observação: 4 visitas sorteadas de 3 horas, com contagem a cada 30 minutos</t>
+          <t>Contagem única por unidade</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -944,7 +944,7 @@
       <c r="A16" s="5" t="n"/>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Mesas ocupadas</t>
+          <t>Mesas ocupadas (quando visíveis de fora)</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Formulário de observação: 4 visitas sorteadas de 3 horas, com contagem a cada 30 minutos</t>
+          <t>Formulário de observação, do lado de fora: 2 visitas sorteadas e 2 de retorno 15 dias depois, com contagem a cada 30 minutos</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Formulário de observação: 4 visitas sorteadas de 3 horas, com contagem a cada 30 minutos</t>
+          <t>Formulário de observação, do lado de fora: 2 visitas sorteadas e 2 de retorno 15 dias depois, no registro de entrada</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Formulário de observação: horário de chegada e saída de cada grupo nas mesmas visitas</t>
+          <t>Formulário de observação, do lado de fora: 2 visitas sorteadas e 2 de retorno 15 dias depois: horário de entrada e saída de cada grupo</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1034,7 +1034,7 @@
       <c r="A19" s="5" t="n"/>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>População por capital</t>
+          <t>População de Salvador, por bairro</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Dimensionar o público potencial</t>
+          <t>Dimensionar o público potencial e escolher o bairro</t>
         </is>
       </c>
       <c r="G19" s="2" t="n"/>
@@ -1064,7 +1064,7 @@
       <c r="A20" s="5" t="n"/>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Renda por capital</t>
+          <t>Renda em Salvador</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Dimensionar o mercado e comparar o poder de compra entre capitais</t>
+          <t>Dimensionar o mercado e comparar o poder de compra com as demais metrópoles</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Horários mais movimentados (taxa de ocupação por turno)</t>
+          <t>Horários mais movimentados (pessoas por hora)</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Formulário de observação: 4 visitas sorteadas de 3 horas, com contagem a cada 30 minutos</t>
+          <t>Formulário de observação, do lado de fora: 2 visitas sorteadas e 2 de retorno 15 dias depois</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Localizar os concorrentes e atribuir capital e bairro</t>
+          <t>Localizar os concorrentes e atribuir metrópole e bairro</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Salário de admissão por ocupação e capital</t>
+          <t>Salário de admissão por ocupação em Salvador</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1436,7 +1436,7 @@
       <c r="A32" s="5" t="n"/>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Aluguel comercial por m²</t>
+          <t>Aluguel comercial por m² em Salvador</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">

</xml_diff>